<commit_message>
qa-agent import cases: a case with no id gets the project's next free id
The team's own ids are never renumbered. A case without one gets the next
number with the project's prefix (case_id_prefix, default TC), worked out after
every file is read; imported again, it keeps that id. In the example, the
id-less Postman request is now TC042, and the team's sheets carry tags.
</commit_message>
<xml_diff>
--- a/examples/bookings-team/existing/booking_cases.xlsx
+++ b/examples/bookings-team/existing/booking_cases.xlsx
@@ -517,7 +517,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>smoke, crud</t>
+        </is>
+      </c>
       <c r="F2" t="n">
         <v>1</v>
       </c>
@@ -622,7 +626,11 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>crud</t>
+        </is>
+      </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
@@ -712,7 +720,11 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>crud, negative</t>
+        </is>
+      </c>
       <c r="F8" t="n">
         <v>1</v>
       </c>

</xml_diff>